<commit_message>
FII/DII: add 10 Jun 2026 (NSE) — cloud cron missed it (NSE 403s GitHub IPs, Groww 502, MC parse fail)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I548"/>
+  <dimension ref="A1:I549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +507,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -977,7 +977,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3765,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3906,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4313,7 +4313,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4689,7 +4689,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5065,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5535,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5582,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5817,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6052,7 +6052,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6240,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6287,7 +6287,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6381,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6428,7 +6428,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6569,7 +6569,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6616,7 +6616,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6710,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6757,7 +6757,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6804,7 +6804,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6851,7 +6851,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6898,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6945,7 +6945,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7039,7 +7039,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7133,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7227,7 +7227,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7274,7 +7274,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7321,7 +7321,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7368,7 +7368,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7462,7 +7462,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7509,7 +7509,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7603,7 +7603,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7650,7 +7650,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7697,7 +7697,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7791,7 +7791,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7877,7 +7877,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7924,7 +7924,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -7963,7 +7963,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8104,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8245,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8292,7 +8292,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8339,7 +8339,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8386,7 +8386,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8480,7 +8480,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8527,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8574,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8621,7 +8621,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8715,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8809,7 +8809,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8856,7 +8856,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8903,7 +8903,7 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8997,7 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9044,7 +9044,7 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9091,7 +9091,7 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9326,7 +9326,7 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9373,7 +9373,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9412,7 +9412,7 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9459,7 +9459,7 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9506,7 +9506,7 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9553,7 +9553,7 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9600,7 +9600,7 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9647,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9694,7 +9694,7 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9788,7 +9788,7 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9882,7 +9882,7 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9929,7 +9929,7 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -9976,7 +9976,7 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10070,7 +10070,7 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10117,7 +10117,7 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10164,7 +10164,7 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10211,7 +10211,7 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10305,7 +10305,7 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10352,7 +10352,7 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10446,7 +10446,7 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10540,7 +10540,7 @@
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10634,7 +10634,7 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10681,7 +10681,7 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10728,7 +10728,7 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10775,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10869,7 +10869,7 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10916,7 +10916,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -10963,7 +10963,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11010,7 +11010,7 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11057,7 +11057,7 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11151,7 +11151,7 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11198,7 +11198,7 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11245,7 +11245,7 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11339,7 +11339,7 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11386,7 +11386,7 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11433,7 +11433,7 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11480,7 +11480,7 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11527,7 +11527,7 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11574,7 +11574,7 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11621,7 +11621,7 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11668,7 +11668,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11715,7 +11715,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11809,7 +11809,7 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11856,7 +11856,7 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11903,7 +11903,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11950,7 +11950,7 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -11997,7 +11997,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12044,7 +12044,7 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12091,7 +12091,7 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12138,7 +12138,7 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12185,7 +12185,7 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12232,7 +12232,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12279,7 +12279,7 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12326,7 +12326,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12365,7 +12365,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12412,7 +12412,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12506,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12553,7 +12553,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12600,7 +12600,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12694,7 +12694,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12741,7 +12741,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12788,7 +12788,7 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12882,7 +12882,7 @@
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12929,7 +12929,7 @@
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -12968,7 +12968,7 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13015,7 +13015,7 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13062,7 +13062,7 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13109,7 +13109,7 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13156,7 +13156,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13203,7 +13203,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13250,7 +13250,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13297,7 +13297,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13344,7 +13344,7 @@
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13391,7 +13391,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13438,7 +13438,7 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13485,7 +13485,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13532,7 +13532,7 @@
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13579,7 +13579,7 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13626,7 +13626,7 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13673,7 +13673,7 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13720,7 +13720,7 @@
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13767,7 +13767,7 @@
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13814,7 +13814,7 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13861,7 +13861,7 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13908,7 +13908,7 @@
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -13955,7 +13955,7 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14002,7 +14002,7 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14096,7 +14096,7 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14143,7 +14143,7 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14190,7 +14190,7 @@
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14237,7 +14237,7 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14284,7 +14284,7 @@
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14331,7 +14331,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14378,7 +14378,7 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14425,7 +14425,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14472,7 +14472,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14519,7 +14519,7 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14566,7 +14566,7 @@
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14613,7 +14613,7 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14660,7 +14660,7 @@
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14707,7 +14707,7 @@
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14754,7 +14754,7 @@
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14848,7 +14848,7 @@
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14895,7 +14895,7 @@
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -14989,7 +14989,7 @@
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15036,7 +15036,7 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15083,7 +15083,7 @@
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15130,7 +15130,7 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15177,7 +15177,7 @@
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15224,7 +15224,7 @@
       </c>
       <c r="I317" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15271,7 +15271,7 @@
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15318,7 +15318,7 @@
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15365,7 +15365,7 @@
       </c>
       <c r="I320" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15412,7 +15412,7 @@
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15459,7 +15459,7 @@
       </c>
       <c r="I322" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15506,7 +15506,7 @@
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15553,7 +15553,7 @@
       </c>
       <c r="I324" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15600,7 +15600,7 @@
       </c>
       <c r="I325" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15647,7 +15647,7 @@
       </c>
       <c r="I326" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15694,7 +15694,7 @@
       </c>
       <c r="I327" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15741,7 +15741,7 @@
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15788,7 +15788,7 @@
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15835,7 +15835,7 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15882,7 +15882,7 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15929,7 +15929,7 @@
       </c>
       <c r="I332" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -15976,7 +15976,7 @@
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16023,7 +16023,7 @@
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16070,7 +16070,7 @@
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16117,7 +16117,7 @@
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16164,7 +16164,7 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16211,7 +16211,7 @@
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16258,7 +16258,7 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16305,7 +16305,7 @@
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16352,7 +16352,7 @@
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16399,7 +16399,7 @@
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16446,7 +16446,7 @@
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16493,7 +16493,7 @@
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16540,7 +16540,7 @@
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16587,7 +16587,7 @@
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16634,7 +16634,7 @@
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16681,7 +16681,7 @@
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16728,7 +16728,7 @@
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16775,7 +16775,7 @@
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16822,7 +16822,7 @@
       </c>
       <c r="I351" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16869,7 +16869,7 @@
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16916,7 +16916,7 @@
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -16963,7 +16963,7 @@
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17010,7 +17010,7 @@
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17057,7 +17057,7 @@
       </c>
       <c r="I356" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17104,7 +17104,7 @@
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17151,7 +17151,7 @@
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17198,7 +17198,7 @@
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17245,7 +17245,7 @@
       </c>
       <c r="I360" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17292,7 +17292,7 @@
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17339,7 +17339,7 @@
       </c>
       <c r="I362" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17386,7 +17386,7 @@
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17433,7 +17433,7 @@
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17480,7 +17480,7 @@
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17527,7 +17527,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17574,7 +17574,7 @@
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17621,7 +17621,7 @@
       </c>
       <c r="I368" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17668,7 +17668,7 @@
       </c>
       <c r="I369" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17715,7 +17715,7 @@
       </c>
       <c r="I370" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17762,7 +17762,7 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17809,7 +17809,7 @@
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17856,7 +17856,7 @@
       </c>
       <c r="I373" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="I374" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17950,7 +17950,7 @@
       </c>
       <c r="I375" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -17997,7 +17997,7 @@
       </c>
       <c r="I376" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18044,7 +18044,7 @@
       </c>
       <c r="I377" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18091,7 +18091,7 @@
       </c>
       <c r="I378" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18138,7 +18138,7 @@
       </c>
       <c r="I379" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18185,7 +18185,7 @@
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18232,7 +18232,7 @@
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18279,7 +18279,7 @@
       </c>
       <c r="I382" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18326,7 +18326,7 @@
       </c>
       <c r="I383" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18373,7 +18373,7 @@
       </c>
       <c r="I384" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18420,7 +18420,7 @@
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18467,7 +18467,7 @@
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18514,7 +18514,7 @@
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18561,7 +18561,7 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18608,7 +18608,7 @@
       </c>
       <c r="I389" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18655,7 +18655,7 @@
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18702,7 +18702,7 @@
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18749,7 +18749,7 @@
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18796,7 +18796,7 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18843,7 +18843,7 @@
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18890,7 +18890,7 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18937,7 +18937,7 @@
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -18984,7 +18984,7 @@
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19031,7 +19031,7 @@
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19078,7 +19078,7 @@
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19125,7 +19125,7 @@
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19172,7 +19172,7 @@
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19219,7 +19219,7 @@
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19266,7 +19266,7 @@
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19313,7 +19313,7 @@
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19360,7 +19360,7 @@
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19407,7 +19407,7 @@
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19454,7 +19454,7 @@
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19501,7 +19501,7 @@
       </c>
       <c r="I408" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19548,7 +19548,7 @@
       </c>
       <c r="I409" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19595,7 +19595,7 @@
       </c>
       <c r="I410" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19642,7 +19642,7 @@
       </c>
       <c r="I411" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19689,7 +19689,7 @@
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19736,7 +19736,7 @@
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19783,7 +19783,7 @@
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19830,7 +19830,7 @@
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19877,7 +19877,7 @@
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19924,7 +19924,7 @@
       </c>
       <c r="I417" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19971,7 @@
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20018,7 +20018,7 @@
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20065,7 +20065,7 @@
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20112,7 +20112,7 @@
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20159,7 @@
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20206,7 +20206,7 @@
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20253,7 +20253,7 @@
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20300,7 +20300,7 @@
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20347,7 +20347,7 @@
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20394,7 +20394,7 @@
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20441,7 +20441,7 @@
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20488,7 +20488,7 @@
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20535,7 +20535,7 @@
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20582,7 +20582,7 @@
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20629,7 +20629,7 @@
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20676,7 +20676,7 @@
       </c>
       <c r="I433" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20723,7 +20723,7 @@
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20770,7 +20770,7 @@
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20817,7 +20817,7 @@
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20864,7 +20864,7 @@
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20911,7 +20911,7 @@
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -20958,7 +20958,7 @@
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21005,7 +21005,7 @@
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21052,7 +21052,7 @@
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21099,7 +21099,7 @@
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21193,7 +21193,7 @@
       </c>
       <c r="I444" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21240,7 +21240,7 @@
       </c>
       <c r="I445" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21287,7 +21287,7 @@
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21334,7 +21334,7 @@
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21381,7 +21381,7 @@
       </c>
       <c r="I448" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21428,7 +21428,7 @@
       </c>
       <c r="I449" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21475,7 +21475,7 @@
       </c>
       <c r="I450" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21522,7 +21522,7 @@
       </c>
       <c r="I451" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21569,7 +21569,7 @@
       </c>
       <c r="I452" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21616,7 +21616,7 @@
       </c>
       <c r="I453" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21663,7 +21663,7 @@
       </c>
       <c r="I454" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21710,7 +21710,7 @@
       </c>
       <c r="I455" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21757,7 +21757,7 @@
       </c>
       <c r="I456" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21804,7 +21804,7 @@
       </c>
       <c r="I457" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21851,7 +21851,7 @@
       </c>
       <c r="I458" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21898,7 +21898,7 @@
       </c>
       <c r="I459" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21945,7 +21945,7 @@
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -21992,7 +21992,7 @@
       </c>
       <c r="I461" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22039,7 +22039,7 @@
       </c>
       <c r="I462" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22086,7 +22086,7 @@
       </c>
       <c r="I463" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22133,7 +22133,7 @@
       </c>
       <c r="I464" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22180,7 +22180,7 @@
       </c>
       <c r="I465" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22227,7 +22227,7 @@
       </c>
       <c r="I466" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22274,7 +22274,7 @@
       </c>
       <c r="I467" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22321,7 +22321,7 @@
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22368,7 +22368,7 @@
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22415,7 +22415,7 @@
       </c>
       <c r="I470" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22462,7 +22462,7 @@
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22509,7 +22509,7 @@
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22556,7 +22556,7 @@
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22603,7 +22603,7 @@
       </c>
       <c r="I474" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22650,7 +22650,7 @@
       </c>
       <c r="I475" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22697,7 +22697,7 @@
       </c>
       <c r="I476" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22744,7 +22744,7 @@
       </c>
       <c r="I477" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22791,7 +22791,7 @@
       </c>
       <c r="I478" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22838,7 +22838,7 @@
       </c>
       <c r="I479" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22885,7 +22885,7 @@
       </c>
       <c r="I480" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22932,7 +22932,7 @@
       </c>
       <c r="I481" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -22979,7 +22979,7 @@
       </c>
       <c r="I482" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23026,7 +23026,7 @@
       </c>
       <c r="I483" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23073,7 +23073,7 @@
       </c>
       <c r="I484" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23120,7 +23120,7 @@
       </c>
       <c r="I485" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23167,7 +23167,7 @@
       </c>
       <c r="I486" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23214,7 +23214,7 @@
       </c>
       <c r="I487" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23261,7 +23261,7 @@
       </c>
       <c r="I488" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23308,7 +23308,7 @@
       </c>
       <c r="I489" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23355,7 +23355,7 @@
       </c>
       <c r="I490" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23402,7 +23402,7 @@
       </c>
       <c r="I491" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23449,7 +23449,7 @@
       </c>
       <c r="I492" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23496,7 +23496,7 @@
       </c>
       <c r="I493" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23543,7 +23543,7 @@
       </c>
       <c r="I494" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23590,7 +23590,7 @@
       </c>
       <c r="I495" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23637,7 +23637,7 @@
       </c>
       <c r="I496" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23684,7 +23684,7 @@
       </c>
       <c r="I497" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23731,7 +23731,7 @@
       </c>
       <c r="I498" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23778,7 +23778,7 @@
       </c>
       <c r="I499" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23825,7 +23825,7 @@
       </c>
       <c r="I500" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23872,7 +23872,7 @@
       </c>
       <c r="I501" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23919,7 +23919,7 @@
       </c>
       <c r="I502" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -23966,7 +23966,7 @@
       </c>
       <c r="I503" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24013,7 +24013,7 @@
       </c>
       <c r="I504" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24060,7 +24060,7 @@
       </c>
       <c r="I505" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24107,7 +24107,7 @@
       </c>
       <c r="I506" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24154,7 +24154,7 @@
       </c>
       <c r="I507" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24201,7 +24201,7 @@
       </c>
       <c r="I508" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24248,7 +24248,7 @@
       </c>
       <c r="I509" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24295,7 +24295,7 @@
       </c>
       <c r="I510" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24342,7 +24342,7 @@
       </c>
       <c r="I511" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24389,7 +24389,7 @@
       </c>
       <c r="I512" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24436,7 +24436,7 @@
       </c>
       <c r="I513" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24483,7 +24483,7 @@
       </c>
       <c r="I514" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24530,7 +24530,7 @@
       </c>
       <c r="I515" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24577,7 +24577,7 @@
       </c>
       <c r="I516" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
       </c>
       <c r="I517" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24671,7 +24671,7 @@
       </c>
       <c r="I518" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24718,7 +24718,7 @@
       </c>
       <c r="I519" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24765,7 +24765,7 @@
       </c>
       <c r="I520" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24812,7 +24812,7 @@
       </c>
       <c r="I521" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24859,7 +24859,7 @@
       </c>
       <c r="I522" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24906,7 +24906,7 @@
       </c>
       <c r="I523" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -24953,7 +24953,7 @@
       </c>
       <c r="I524" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25000,7 +25000,7 @@
       </c>
       <c r="I525" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25047,7 +25047,7 @@
       </c>
       <c r="I526" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25094,7 +25094,7 @@
       </c>
       <c r="I527" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25141,7 +25141,7 @@
       </c>
       <c r="I528" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25188,7 +25188,7 @@
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25235,7 +25235,7 @@
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25282,7 +25282,7 @@
       </c>
       <c r="I531" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25329,7 +25329,7 @@
       </c>
       <c r="I532" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25376,7 +25376,7 @@
       </c>
       <c r="I533" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25423,7 +25423,7 @@
       </c>
       <c r="I534" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25470,7 +25470,7 @@
       </c>
       <c r="I535" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25517,7 +25517,7 @@
       </c>
       <c r="I536" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25564,7 +25564,7 @@
       </c>
       <c r="I537" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25611,7 +25611,7 @@
       </c>
       <c r="I538" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25658,7 +25658,7 @@
       </c>
       <c r="I539" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25705,7 +25705,7 @@
       </c>
       <c r="I540" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25752,7 +25752,7 @@
       </c>
       <c r="I541" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25799,7 +25799,7 @@
       </c>
       <c r="I542" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25846,7 +25846,7 @@
       </c>
       <c r="I543" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25893,7 +25893,7 @@
       </c>
       <c r="I544" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25940,7 +25940,7 @@
       </c>
       <c r="I545" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -25987,7 +25987,7 @@
       </c>
       <c r="I546" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -26034,7 +26034,7 @@
       </c>
       <c r="I547" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
         </is>
       </c>
     </row>
@@ -26081,7 +26081,54 @@
       </c>
       <c r="I548" t="inlineStr">
         <is>
-          <t>final</t>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>14047.79</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>16172.77</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>-2124.98</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>17396.4</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>14272.45</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>3123.95</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>provisional</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-09)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I610"/>
+  <dimension ref="A1:I611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28994,6 +28994,53 @@
         </is>
       </c>
       <c r="I610" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>11704.84</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>11828.03</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>-123.19</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>14678.53</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>13328.89</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>1349.64</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-10)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I611"/>
+  <dimension ref="A1:I612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29041,6 +29041,53 @@
         </is>
       </c>
       <c r="I611" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>16392.9</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>16975.89</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>-582.99</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>18130.76</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>16621.72</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>1509.04</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>